<commit_message>
formatar planilha e mostrar ao Leandro
</commit_message>
<xml_diff>
--- a/manutenção/modelo planilha auxiliar indicadores.xlsx
+++ b/manutenção/modelo planilha auxiliar indicadores.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11715" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11715"/>
   </bookViews>
   <sheets>
     <sheet name="PLANILHA" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="207">
   <si>
     <t>FILIAL</t>
   </si>
@@ -810,14 +810,14 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1152,14 +1152,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J159"/>
+  <dimension ref="A1:J317"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" customWidth="1"/>
     <col min="2" max="2" width="19.42578125" customWidth="1"/>
     <col min="3" max="3" width="12.7109375" customWidth="1"/>
     <col min="4" max="4" width="11.85546875" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.5703125" customWidth="1"/>
     <col min="7" max="7" width="13.7109375" customWidth="1"/>
     <col min="8" max="8" width="22.42578125" customWidth="1"/>
@@ -3884,6 +3884,1270 @@
       </c>
       <c r="H159">
         <v>1</v>
+      </c>
+    </row>
+    <row r="160" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D160" t="s">
+        <v>147</v>
+      </c>
+      <c r="E160" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="161" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D161" t="s">
+        <v>148</v>
+      </c>
+      <c r="E161" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="162" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D162" t="s">
+        <v>149</v>
+      </c>
+      <c r="E162" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="163" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D163" t="s">
+        <v>150</v>
+      </c>
+      <c r="E163" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="164" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D164" t="s">
+        <v>151</v>
+      </c>
+      <c r="E164" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="165" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D165" t="s">
+        <v>152</v>
+      </c>
+      <c r="E165" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="166" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D166" t="s">
+        <v>153</v>
+      </c>
+      <c r="E166" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="167" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D167" t="s">
+        <v>154</v>
+      </c>
+      <c r="E167" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="168" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D168" t="s">
+        <v>155</v>
+      </c>
+      <c r="E168" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="169" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D169" t="s">
+        <v>156</v>
+      </c>
+      <c r="E169" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="170" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D170" t="s">
+        <v>157</v>
+      </c>
+      <c r="E170" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="171" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D171" t="s">
+        <v>158</v>
+      </c>
+      <c r="E171" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="172" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D172" t="s">
+        <v>159</v>
+      </c>
+      <c r="E172" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="173" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D173" t="s">
+        <v>160</v>
+      </c>
+      <c r="E173" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="174" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D174" t="s">
+        <v>161</v>
+      </c>
+      <c r="E174" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="175" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D175" t="s">
+        <v>162</v>
+      </c>
+      <c r="E175" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="176" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D176" t="s">
+        <v>163</v>
+      </c>
+      <c r="E176" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="177" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D177" t="s">
+        <v>164</v>
+      </c>
+      <c r="E177" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="178" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D178" t="s">
+        <v>165</v>
+      </c>
+      <c r="E178" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="179" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D179" t="s">
+        <v>166</v>
+      </c>
+      <c r="E179" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="180" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D180" t="s">
+        <v>167</v>
+      </c>
+      <c r="E180" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="181" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D181" t="s">
+        <v>168</v>
+      </c>
+      <c r="E181" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="182" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D182" t="s">
+        <v>169</v>
+      </c>
+      <c r="E182" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="183" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D183" t="s">
+        <v>170</v>
+      </c>
+      <c r="E183" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="184" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D184" t="s">
+        <v>171</v>
+      </c>
+      <c r="E184" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="185" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D185" t="s">
+        <v>172</v>
+      </c>
+      <c r="E185" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="186" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D186" t="s">
+        <v>173</v>
+      </c>
+      <c r="E186" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="187" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D187" t="s">
+        <v>174</v>
+      </c>
+      <c r="E187" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="188" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D188" t="s">
+        <v>175</v>
+      </c>
+      <c r="E188" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="189" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D189" t="s">
+        <v>176</v>
+      </c>
+      <c r="E189" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="190" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D190" t="s">
+        <v>177</v>
+      </c>
+      <c r="E190" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="191" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D191" t="s">
+        <v>178</v>
+      </c>
+      <c r="E191" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="192" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D192" t="s">
+        <v>179</v>
+      </c>
+      <c r="E192" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="193" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D193" t="s">
+        <v>180</v>
+      </c>
+      <c r="E193" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="194" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D194" t="s">
+        <v>181</v>
+      </c>
+      <c r="E194" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="195" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D195" t="s">
+        <v>182</v>
+      </c>
+      <c r="E195" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="196" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D196" t="s">
+        <v>183</v>
+      </c>
+      <c r="E196" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="197" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D197" t="s">
+        <v>184</v>
+      </c>
+      <c r="E197" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="198" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D198" t="s">
+        <v>185</v>
+      </c>
+      <c r="E198" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="199" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D199" t="s">
+        <v>186</v>
+      </c>
+      <c r="E199" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="200" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D200" t="s">
+        <v>187</v>
+      </c>
+      <c r="E200" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="201" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D201" t="s">
+        <v>188</v>
+      </c>
+      <c r="E201" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="202" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D202" t="s">
+        <v>189</v>
+      </c>
+      <c r="E202" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="203" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D203" t="s">
+        <v>190</v>
+      </c>
+      <c r="E203" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="204" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D204" t="s">
+        <v>191</v>
+      </c>
+      <c r="E204" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="205" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D205" t="s">
+        <v>192</v>
+      </c>
+      <c r="E205" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="206" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D206" t="s">
+        <v>193</v>
+      </c>
+      <c r="E206" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="207" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D207" t="s">
+        <v>194</v>
+      </c>
+      <c r="E207" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="208" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D208" t="s">
+        <v>195</v>
+      </c>
+      <c r="E208" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="209" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D209" t="s">
+        <v>196</v>
+      </c>
+      <c r="E209" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="210" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D210" t="s">
+        <v>197</v>
+      </c>
+      <c r="E210" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="211" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D211" t="s">
+        <v>198</v>
+      </c>
+      <c r="E211" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="212" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D212" t="s">
+        <v>199</v>
+      </c>
+      <c r="E212" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="213" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D213" t="s">
+        <v>200</v>
+      </c>
+      <c r="E213" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="214" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D214" t="s">
+        <v>201</v>
+      </c>
+      <c r="E214" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="215" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D215" t="s">
+        <v>202</v>
+      </c>
+      <c r="E215" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="216" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D216" t="s">
+        <v>203</v>
+      </c>
+      <c r="E216" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="217" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D217" t="s">
+        <v>144</v>
+      </c>
+      <c r="E217" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="218" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D218" t="s">
+        <v>145</v>
+      </c>
+      <c r="E218" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="219" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D219" t="s">
+        <v>146</v>
+      </c>
+      <c r="E219" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="220" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D220" t="s">
+        <v>20</v>
+      </c>
+      <c r="E220" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="221" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D221" t="s">
+        <v>47</v>
+      </c>
+      <c r="E221" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="222" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D222" t="s">
+        <v>48</v>
+      </c>
+      <c r="E222" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="223" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D223" t="s">
+        <v>49</v>
+      </c>
+      <c r="E223" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="224" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D224" t="s">
+        <v>50</v>
+      </c>
+      <c r="E224" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="225" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D225" t="s">
+        <v>51</v>
+      </c>
+      <c r="E225" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="226" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D226" t="s">
+        <v>52</v>
+      </c>
+      <c r="E226" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="227" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D227" t="s">
+        <v>53</v>
+      </c>
+      <c r="E227" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="228" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D228" t="s">
+        <v>54</v>
+      </c>
+      <c r="E228" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="229" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D229" t="s">
+        <v>55</v>
+      </c>
+      <c r="E229" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="230" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D230" t="s">
+        <v>56</v>
+      </c>
+      <c r="E230" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="231" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D231" t="s">
+        <v>57</v>
+      </c>
+      <c r="E231" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="232" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D232" t="s">
+        <v>58</v>
+      </c>
+      <c r="E232" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="233" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D233" t="s">
+        <v>59</v>
+      </c>
+      <c r="E233" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="234" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D234" t="s">
+        <v>60</v>
+      </c>
+      <c r="E234" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="235" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D235" t="s">
+        <v>61</v>
+      </c>
+      <c r="E235" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="236" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D236" t="s">
+        <v>62</v>
+      </c>
+      <c r="E236" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="237" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D237" t="s">
+        <v>63</v>
+      </c>
+      <c r="E237" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="238" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D238" t="s">
+        <v>64</v>
+      </c>
+      <c r="E238" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="239" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D239" t="s">
+        <v>65</v>
+      </c>
+      <c r="E239" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="240" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D240" t="s">
+        <v>66</v>
+      </c>
+      <c r="E240" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="241" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D241" t="s">
+        <v>67</v>
+      </c>
+      <c r="E241" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="242" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D242" t="s">
+        <v>68</v>
+      </c>
+      <c r="E242" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="243" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D243" t="s">
+        <v>69</v>
+      </c>
+      <c r="E243" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="244" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D244" t="s">
+        <v>70</v>
+      </c>
+      <c r="E244" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="245" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D245" t="s">
+        <v>71</v>
+      </c>
+      <c r="E245" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="246" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D246" t="s">
+        <v>72</v>
+      </c>
+      <c r="E246" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="247" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D247" t="s">
+        <v>73</v>
+      </c>
+      <c r="E247" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="248" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D248" t="s">
+        <v>74</v>
+      </c>
+      <c r="E248" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="249" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D249" t="s">
+        <v>75</v>
+      </c>
+      <c r="E249" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="250" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D250" t="s">
+        <v>76</v>
+      </c>
+      <c r="E250" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="251" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D251" t="s">
+        <v>77</v>
+      </c>
+      <c r="E251" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="252" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D252" t="s">
+        <v>78</v>
+      </c>
+      <c r="E252" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="253" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D253" t="s">
+        <v>79</v>
+      </c>
+      <c r="E253" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="254" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D254" t="s">
+        <v>80</v>
+      </c>
+      <c r="E254" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="255" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D255" t="s">
+        <v>81</v>
+      </c>
+      <c r="E255" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="256" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D256" t="s">
+        <v>82</v>
+      </c>
+      <c r="E256" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="257" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D257" t="s">
+        <v>83</v>
+      </c>
+      <c r="E257" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="258" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D258" t="s">
+        <v>84</v>
+      </c>
+      <c r="E258" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="259" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D259" t="s">
+        <v>85</v>
+      </c>
+      <c r="E259" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="260" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D260" t="s">
+        <v>86</v>
+      </c>
+      <c r="E260" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="261" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D261" t="s">
+        <v>87</v>
+      </c>
+      <c r="E261" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="262" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D262" t="s">
+        <v>88</v>
+      </c>
+      <c r="E262" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="263" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D263" t="s">
+        <v>89</v>
+      </c>
+      <c r="E263" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="264" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D264" t="s">
+        <v>90</v>
+      </c>
+      <c r="E264" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="265" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D265" t="s">
+        <v>91</v>
+      </c>
+      <c r="E265" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="266" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D266" t="s">
+        <v>92</v>
+      </c>
+      <c r="E266" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="267" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D267" t="s">
+        <v>93</v>
+      </c>
+      <c r="E267" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="268" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D268" t="s">
+        <v>94</v>
+      </c>
+      <c r="E268" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="269" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D269" t="s">
+        <v>95</v>
+      </c>
+      <c r="E269" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="270" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D270" t="s">
+        <v>96</v>
+      </c>
+      <c r="E270" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="271" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D271" t="s">
+        <v>97</v>
+      </c>
+      <c r="E271" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="272" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D272" t="s">
+        <v>98</v>
+      </c>
+      <c r="E272" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="273" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D273" t="s">
+        <v>99</v>
+      </c>
+      <c r="E273" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="274" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D274" t="s">
+        <v>100</v>
+      </c>
+      <c r="E274" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="275" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D275" t="s">
+        <v>101</v>
+      </c>
+      <c r="E275" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="276" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D276" t="s">
+        <v>102</v>
+      </c>
+      <c r="E276" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="277" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D277" t="s">
+        <v>103</v>
+      </c>
+      <c r="E277" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="278" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D278" t="s">
+        <v>104</v>
+      </c>
+      <c r="E278" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="279" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D279" t="s">
+        <v>105</v>
+      </c>
+      <c r="E279" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="280" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D280" t="s">
+        <v>106</v>
+      </c>
+      <c r="E280" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="281" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D281" t="s">
+        <v>107</v>
+      </c>
+      <c r="E281" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="282" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D282" t="s">
+        <v>108</v>
+      </c>
+      <c r="E282" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="283" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D283" t="s">
+        <v>109</v>
+      </c>
+      <c r="E283" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="284" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D284" t="s">
+        <v>110</v>
+      </c>
+      <c r="E284" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="285" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D285" t="s">
+        <v>111</v>
+      </c>
+      <c r="E285" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="286" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D286" t="s">
+        <v>112</v>
+      </c>
+      <c r="E286" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="287" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D287" t="s">
+        <v>113</v>
+      </c>
+      <c r="E287" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="288" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D288" t="s">
+        <v>114</v>
+      </c>
+      <c r="E288" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="289" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D289" t="s">
+        <v>115</v>
+      </c>
+      <c r="E289" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="290" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D290" t="s">
+        <v>116</v>
+      </c>
+      <c r="E290" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="291" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D291" t="s">
+        <v>117</v>
+      </c>
+      <c r="E291" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="292" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D292" t="s">
+        <v>118</v>
+      </c>
+      <c r="E292" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="293" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D293" t="s">
+        <v>119</v>
+      </c>
+      <c r="E293" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="294" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D294" t="s">
+        <v>120</v>
+      </c>
+      <c r="E294" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="295" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D295" t="s">
+        <v>121</v>
+      </c>
+      <c r="E295" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="296" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D296" t="s">
+        <v>122</v>
+      </c>
+      <c r="E296" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="297" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D297" t="s">
+        <v>123</v>
+      </c>
+      <c r="E297" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="298" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D298" t="s">
+        <v>124</v>
+      </c>
+      <c r="E298" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="299" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D299" t="s">
+        <v>125</v>
+      </c>
+      <c r="E299" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="300" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D300" t="s">
+        <v>126</v>
+      </c>
+      <c r="E300" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="301" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D301" t="s">
+        <v>127</v>
+      </c>
+      <c r="E301" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="302" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D302" t="s">
+        <v>128</v>
+      </c>
+      <c r="E302" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="303" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D303" t="s">
+        <v>129</v>
+      </c>
+      <c r="E303" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="304" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D304" t="s">
+        <v>130</v>
+      </c>
+      <c r="E304" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="305" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D305" t="s">
+        <v>131</v>
+      </c>
+      <c r="E305" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="306" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D306" t="s">
+        <v>132</v>
+      </c>
+      <c r="E306" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="307" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D307" t="s">
+        <v>133</v>
+      </c>
+      <c r="E307" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="308" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D308" t="s">
+        <v>134</v>
+      </c>
+      <c r="E308" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="309" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D309" t="s">
+        <v>135</v>
+      </c>
+      <c r="E309" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="310" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D310" t="s">
+        <v>136</v>
+      </c>
+      <c r="E310" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="311" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D311" t="s">
+        <v>137</v>
+      </c>
+      <c r="E311" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="312" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D312" t="s">
+        <v>138</v>
+      </c>
+      <c r="E312" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="313" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D313" t="s">
+        <v>139</v>
+      </c>
+      <c r="E313" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="314" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D314" t="s">
+        <v>140</v>
+      </c>
+      <c r="E314" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="315" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D315" t="s">
+        <v>141</v>
+      </c>
+      <c r="E315" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="316" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D316" t="s">
+        <v>142</v>
+      </c>
+      <c r="E316" s="24">
+        <v>45079</v>
+      </c>
+    </row>
+    <row r="317" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D317" t="s">
+        <v>143</v>
+      </c>
+      <c r="E317" s="24">
+        <v>45079</v>
       </c>
     </row>
   </sheetData>
@@ -3940,12 +5204,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
       <c r="E1" s="5" t="s">
         <v>30</v>
       </c>
@@ -3962,12 +5226,12 @@
         <f>'[1]ATA REUNIÃO PCM 27.06'!P3</f>
         <v>45104</v>
       </c>
-      <c r="J1" s="27" t="s">
+      <c r="J1" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
       <c r="N1" s="5" t="s">
         <v>30</v>
       </c>
@@ -3977,12 +5241,12 @@
       <c r="P1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="Q1" s="27" t="s">
+      <c r="Q1" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="28"/>
-      <c r="S1" s="28"/>
-      <c r="T1" s="28"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
       <c r="U1" s="6" t="s">
         <v>206</v>
       </c>
@@ -4067,11 +5331,11 @@
       </c>
       <c r="F3" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A3,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G3" s="17">
         <f t="shared" ref="G3" si="0">F3/E3</f>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>38</v>
@@ -4098,7 +5362,7 @@
       <c r="T3" s="25"/>
       <c r="U3" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q3,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V3" s="16">
         <v>8</v>
@@ -4117,11 +5381,11 @@
       </c>
       <c r="F4" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A4,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G4" s="17">
         <f>F4/E4</f>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>39</v>
@@ -4148,7 +5412,7 @@
       <c r="T4" s="25"/>
       <c r="U4" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q4,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V4" s="16">
         <v>8</v>
@@ -4167,11 +5431,11 @@
       </c>
       <c r="F5" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A5,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G5" s="17">
         <f t="shared" ref="G5:G32" si="1">F5/E5</f>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H5" s="18" t="s">
         <v>40</v>
@@ -4198,7 +5462,7 @@
       <c r="T5" s="25"/>
       <c r="U5" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q5,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V5" s="16">
         <v>8</v>
@@ -4217,11 +5481,11 @@
       </c>
       <c r="F6" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A6,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G6" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>41</v>
@@ -4248,7 +5512,7 @@
       <c r="T6" s="25"/>
       <c r="U6" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q6,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V6" s="16">
         <v>8</v>
@@ -4267,11 +5531,11 @@
       </c>
       <c r="F7" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A7,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G7" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>42</v>
@@ -4298,7 +5562,7 @@
       <c r="T7" s="25"/>
       <c r="U7" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q7,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V7" s="16">
         <v>8</v>
@@ -4317,11 +5581,11 @@
       </c>
       <c r="F8" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A8,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G8" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>43</v>
@@ -4348,7 +5612,7 @@
       <c r="T8" s="25"/>
       <c r="U8" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q8,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V8" s="16">
         <v>7</v>
@@ -4367,11 +5631,11 @@
       </c>
       <c r="F9" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A9,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G9" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H9" s="18" t="s">
         <v>44</v>
@@ -4398,7 +5662,7 @@
       <c r="T9" s="25"/>
       <c r="U9" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q9,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V9" s="16">
         <v>5</v>
@@ -4417,11 +5681,11 @@
       </c>
       <c r="F10" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A10,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G10" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H10"/>
       <c r="I10"/>
@@ -4444,7 +5708,7 @@
       <c r="T10" s="25"/>
       <c r="U10" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q10,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V10" s="16">
         <v>5</v>
@@ -4463,11 +5727,11 @@
       </c>
       <c r="F11" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A11,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G11" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H11"/>
       <c r="I11"/>
@@ -4490,7 +5754,7 @@
       <c r="T11" s="25"/>
       <c r="U11" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q11,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V11" s="16">
         <v>5</v>
@@ -4509,11 +5773,11 @@
       </c>
       <c r="F12" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A12,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G12" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H12"/>
       <c r="I12"/>
@@ -4536,7 +5800,7 @@
       <c r="T12" s="25"/>
       <c r="U12" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q12,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V12" s="16">
         <v>5</v>
@@ -4555,11 +5819,11 @@
       </c>
       <c r="F13" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A13,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G13" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H13"/>
       <c r="I13"/>
@@ -4582,7 +5846,7 @@
       <c r="T13" s="25"/>
       <c r="U13" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q13,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V13" s="16">
         <v>5</v>
@@ -4601,11 +5865,11 @@
       </c>
       <c r="F14" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A14,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G14" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H14"/>
       <c r="I14"/>
@@ -4628,7 +5892,7 @@
       <c r="T14" s="25"/>
       <c r="U14" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q14,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V14" s="16">
         <v>5</v>
@@ -4647,11 +5911,11 @@
       </c>
       <c r="F15" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A15,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G15" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="J15" s="25">
         <v>45091</v>
@@ -4672,7 +5936,7 @@
       <c r="T15" s="25"/>
       <c r="U15" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q15,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V15" s="16">
         <v>5</v>
@@ -4691,11 +5955,11 @@
       </c>
       <c r="F16" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A16,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G16" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H16"/>
       <c r="I16"/>
@@ -4718,7 +5982,7 @@
       <c r="T16" s="25"/>
       <c r="U16" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q16,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V16" s="16">
         <v>5</v>
@@ -4737,11 +6001,11 @@
       </c>
       <c r="F17" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A17,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G17" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H17"/>
       <c r="I17"/>
@@ -4764,7 +6028,7 @@
       <c r="T17" s="25"/>
       <c r="U17" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q17,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V17" s="16">
         <v>5</v>
@@ -4783,11 +6047,11 @@
       </c>
       <c r="F18" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A18,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G18" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H18"/>
       <c r="I18"/>
@@ -4810,7 +6074,7 @@
       <c r="T18" s="25"/>
       <c r="U18" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q18,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V18" s="16">
         <v>5</v>
@@ -4829,11 +6093,11 @@
       </c>
       <c r="F19" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A19,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G19" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H19"/>
       <c r="I19"/>
@@ -4856,7 +6120,7 @@
       <c r="T19" s="25"/>
       <c r="U19" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q19,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V19" s="16">
         <v>5</v>
@@ -4875,11 +6139,11 @@
       </c>
       <c r="F20" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A20,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G20" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H20"/>
       <c r="I20"/>
@@ -4902,7 +6166,7 @@
       <c r="T20" s="25"/>
       <c r="U20" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q20,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V20" s="16">
         <v>5</v>
@@ -4921,11 +6185,11 @@
       </c>
       <c r="F21" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A21,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G21" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -4948,7 +6212,7 @@
       <c r="T21" s="25"/>
       <c r="U21" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q21,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V21" s="16">
         <v>5</v>
@@ -4967,11 +6231,11 @@
       </c>
       <c r="F22" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A22,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G22" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H22"/>
       <c r="I22"/>
@@ -4994,7 +6258,7 @@
       <c r="T22" s="25"/>
       <c r="U22" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q22,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V22" s="16">
         <v>5</v>
@@ -5013,11 +6277,11 @@
       </c>
       <c r="F23" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A23,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G23" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H23"/>
       <c r="I23"/>
@@ -5040,7 +6304,7 @@
       <c r="T23" s="25"/>
       <c r="U23" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q23,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V23" s="16">
         <v>6</v>
@@ -5059,11 +6323,11 @@
       </c>
       <c r="F24" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A24,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G24" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
@@ -5086,7 +6350,7 @@
       <c r="T24" s="25"/>
       <c r="U24" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q24,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V24" s="16">
         <v>6</v>
@@ -5105,11 +6369,11 @@
       </c>
       <c r="F25" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A25,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G25" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H25" s="17"/>
       <c r="I25" s="17"/>
@@ -5132,7 +6396,7 @@
       <c r="T25" s="25"/>
       <c r="U25" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q25,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V25" s="16">
         <v>6</v>
@@ -5151,11 +6415,11 @@
       </c>
       <c r="F26" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A26,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G26" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H26" s="17"/>
       <c r="I26" s="17"/>
@@ -5178,7 +6442,7 @@
       <c r="T26" s="25"/>
       <c r="U26" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q26,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V26" s="16">
         <v>6</v>
@@ -5197,11 +6461,11 @@
       </c>
       <c r="F27" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A27,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G27" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H27" s="17"/>
       <c r="I27" s="17"/>
@@ -5224,7 +6488,7 @@
       <c r="T27" s="25"/>
       <c r="U27" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q27,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V27" s="16">
         <v>6</v>
@@ -5243,11 +6507,11 @@
       </c>
       <c r="F28" s="12">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(A28,Tabela1[[DATA]:[DATA]],1),Tabela1[[DISPONIBILIDADE]:[DISPONIBILIDADE]],1)</f>
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G28" s="17">
         <f t="shared" si="1"/>
-        <v>1.8095238095238095</v>
+        <v>0</v>
       </c>
       <c r="H28" s="17"/>
       <c r="I28" s="17"/>
@@ -5270,7 +6534,7 @@
       <c r="T28" s="25"/>
       <c r="U28" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q28,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V28" s="16">
         <v>6</v>
@@ -5307,7 +6571,7 @@
       <c r="T29" s="25"/>
       <c r="U29" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q29,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V29" s="16"/>
     </row>
@@ -5342,7 +6606,7 @@
       <c r="T30" s="25"/>
       <c r="U30" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q30,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V30" s="16"/>
     </row>
@@ -5377,7 +6641,7 @@
       <c r="T31" s="25"/>
       <c r="U31" s="21">
         <f>SUMIFS(Tabela1[DISPONÍVEL],Tabela1[[DATA]:[DATA]],VLOOKUP(Q31,Tabela1[[DATA]:[DATA]],1),Tabela1[[AGUARDANDO PEÇAS]:[AGUARDANDO PEÇAS]],1)</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V31" s="16"/>
     </row>
@@ -5420,11 +6684,11 @@
       </c>
       <c r="F33" s="20">
         <f>SUM(F2:F32)</f>
-        <v>990</v>
+        <v>2</v>
       </c>
       <c r="G33" s="17">
         <f>F33/E33</f>
-        <v>1.746031746031746</v>
+        <v>3.5273368606701938E-3</v>
       </c>
       <c r="H33" s="17"/>
       <c r="I33" s="17"/>
@@ -5454,734 +6718,924 @@
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" s="25"/>
-      <c r="B34" s="26"/>
-      <c r="C34" s="26"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
       <c r="J34" s="25"/>
-      <c r="K34" s="26"/>
-      <c r="L34" s="26"/>
-      <c r="M34" s="26"/>
+      <c r="K34" s="28"/>
+      <c r="L34" s="28"/>
+      <c r="M34" s="28"/>
       <c r="N34" s="21"/>
       <c r="O34" s="21"/>
-      <c r="Q34" s="26"/>
-      <c r="R34" s="26"/>
-      <c r="S34" s="26"/>
-      <c r="T34" s="26"/>
-      <c r="U34" s="26"/>
-      <c r="V34" s="26"/>
+      <c r="Q34" s="28"/>
+      <c r="R34" s="28"/>
+      <c r="S34" s="28"/>
+      <c r="T34" s="28"/>
+      <c r="U34" s="28"/>
+      <c r="V34" s="28"/>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" s="25"/>
-      <c r="B35" s="26"/>
-      <c r="C35" s="26"/>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
-      <c r="F35" s="26"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
       <c r="J35" s="25"/>
-      <c r="K35" s="26"/>
-      <c r="L35" s="26"/>
-      <c r="M35" s="26"/>
+      <c r="K35" s="28"/>
+      <c r="L35" s="28"/>
+      <c r="M35" s="28"/>
       <c r="N35" s="21"/>
       <c r="O35" s="21"/>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" s="25"/>
-      <c r="B36" s="26"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="26"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28"/>
       <c r="H36" s="22"/>
       <c r="I36" s="22"/>
       <c r="J36" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="K36" s="26"/>
-      <c r="L36" s="26"/>
-      <c r="M36" s="26"/>
+      <c r="K36" s="28"/>
+      <c r="L36" s="28"/>
+      <c r="M36" s="28"/>
       <c r="N36" s="21"/>
       <c r="O36" s="21"/>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" s="25"/>
-      <c r="B37" s="26"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28"/>
       <c r="H37" s="23"/>
       <c r="I37" s="23"/>
       <c r="J37" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="K37" s="26"/>
-      <c r="L37" s="26"/>
-      <c r="M37" s="26"/>
+      <c r="K37" s="28"/>
+      <c r="L37" s="28"/>
+      <c r="M37" s="28"/>
       <c r="N37" s="21"/>
       <c r="O37" s="21"/>
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" s="25"/>
-      <c r="B38" s="26"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="26"/>
-      <c r="F38" s="26"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="28"/>
       <c r="J38" s="25"/>
-      <c r="K38" s="26"/>
-      <c r="L38" s="26"/>
-      <c r="M38" s="26"/>
+      <c r="K38" s="28"/>
+      <c r="L38" s="28"/>
+      <c r="M38" s="28"/>
       <c r="N38" s="21"/>
       <c r="O38" s="21"/>
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" s="25"/>
-      <c r="B39" s="26"/>
-      <c r="C39" s="26"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="26"/>
+      <c r="B39" s="28"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="28"/>
+      <c r="E39" s="28"/>
+      <c r="F39" s="28"/>
       <c r="J39" s="25"/>
-      <c r="K39" s="26"/>
-      <c r="L39" s="26"/>
-      <c r="M39" s="26"/>
+      <c r="K39" s="28"/>
+      <c r="L39" s="28"/>
+      <c r="M39" s="28"/>
       <c r="N39" s="21"/>
       <c r="O39" s="21"/>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" s="25"/>
-      <c r="B40" s="26"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="26"/>
-      <c r="F40" s="26"/>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
       <c r="J40" s="25"/>
-      <c r="K40" s="26"/>
-      <c r="L40" s="26"/>
-      <c r="M40" s="26"/>
+      <c r="K40" s="28"/>
+      <c r="L40" s="28"/>
+      <c r="M40" s="28"/>
       <c r="N40" s="21"/>
       <c r="O40" s="21"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" s="25"/>
-      <c r="B41" s="26"/>
-      <c r="C41" s="26"/>
-      <c r="D41" s="26"/>
-      <c r="E41" s="26"/>
-      <c r="F41" s="26"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="28"/>
+      <c r="F41" s="28"/>
       <c r="J41" s="25"/>
-      <c r="K41" s="26"/>
-      <c r="L41" s="26"/>
-      <c r="M41" s="26"/>
+      <c r="K41" s="28"/>
+      <c r="L41" s="28"/>
+      <c r="M41" s="28"/>
       <c r="N41" s="21"/>
       <c r="O41" s="21"/>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" s="25"/>
-      <c r="B42" s="26"/>
-      <c r="C42" s="26"/>
-      <c r="D42" s="26"/>
-      <c r="E42" s="26"/>
-      <c r="F42" s="26"/>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
       <c r="J42" s="25"/>
-      <c r="K42" s="26"/>
-      <c r="L42" s="26"/>
-      <c r="M42" s="26"/>
+      <c r="K42" s="28"/>
+      <c r="L42" s="28"/>
+      <c r="M42" s="28"/>
       <c r="N42" s="21"/>
       <c r="O42" s="21"/>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" s="25"/>
-      <c r="B43" s="26"/>
-      <c r="C43" s="26"/>
-      <c r="D43" s="26"/>
-      <c r="E43" s="26"/>
-      <c r="F43" s="26"/>
+      <c r="B43" s="28"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="28"/>
+      <c r="F43" s="28"/>
       <c r="J43" s="25"/>
-      <c r="K43" s="26"/>
-      <c r="L43" s="26"/>
-      <c r="M43" s="26"/>
+      <c r="K43" s="28"/>
+      <c r="L43" s="28"/>
+      <c r="M43" s="28"/>
       <c r="N43" s="21"/>
       <c r="O43" s="21"/>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" s="25"/>
-      <c r="B44" s="26"/>
-      <c r="C44" s="26"/>
-      <c r="D44" s="26"/>
-      <c r="E44" s="26"/>
-      <c r="F44" s="26"/>
+      <c r="B44" s="28"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="28"/>
       <c r="J44" s="25"/>
-      <c r="K44" s="26"/>
-      <c r="L44" s="26"/>
-      <c r="M44" s="26"/>
+      <c r="K44" s="28"/>
+      <c r="L44" s="28"/>
+      <c r="M44" s="28"/>
       <c r="N44" s="21"/>
       <c r="O44" s="21"/>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" s="25"/>
-      <c r="B45" s="26"/>
-      <c r="C45" s="26"/>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
-      <c r="F45" s="26"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="28"/>
       <c r="J45" s="25"/>
-      <c r="K45" s="26"/>
-      <c r="L45" s="26"/>
-      <c r="M45" s="26"/>
+      <c r="K45" s="28"/>
+      <c r="L45" s="28"/>
+      <c r="M45" s="28"/>
       <c r="N45" s="21"/>
       <c r="O45" s="21"/>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" s="25"/>
-      <c r="B46" s="26"/>
-      <c r="C46" s="26"/>
-      <c r="D46" s="26"/>
-      <c r="E46" s="26"/>
-      <c r="F46" s="26"/>
+      <c r="B46" s="28"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="28"/>
+      <c r="F46" s="28"/>
       <c r="J46" s="25"/>
-      <c r="K46" s="26"/>
-      <c r="L46" s="26"/>
-      <c r="M46" s="26"/>
+      <c r="K46" s="28"/>
+      <c r="L46" s="28"/>
+      <c r="M46" s="28"/>
       <c r="N46" s="21"/>
       <c r="O46" s="21"/>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A47" s="25"/>
-      <c r="B47" s="26"/>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="28"/>
+      <c r="F47" s="28"/>
       <c r="J47" s="25"/>
-      <c r="K47" s="26"/>
-      <c r="L47" s="26"/>
-      <c r="M47" s="26"/>
+      <c r="K47" s="28"/>
+      <c r="L47" s="28"/>
+      <c r="M47" s="28"/>
       <c r="N47" s="21"/>
       <c r="O47" s="21"/>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A48" s="25"/>
-      <c r="B48" s="26"/>
-      <c r="C48" s="26"/>
-      <c r="D48" s="26"/>
-      <c r="E48" s="26"/>
-      <c r="F48" s="26"/>
+      <c r="B48" s="28"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="28"/>
+      <c r="F48" s="28"/>
       <c r="J48" s="25"/>
-      <c r="K48" s="26"/>
-      <c r="L48" s="26"/>
-      <c r="M48" s="26"/>
+      <c r="K48" s="28"/>
+      <c r="L48" s="28"/>
+      <c r="M48" s="28"/>
       <c r="N48" s="21"/>
       <c r="O48" s="21"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="25"/>
-      <c r="B49" s="26"/>
-      <c r="C49" s="26"/>
-      <c r="D49" s="26"/>
-      <c r="E49" s="26"/>
-      <c r="F49" s="26"/>
+      <c r="B49" s="28"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="28"/>
+      <c r="F49" s="28"/>
       <c r="J49" s="25"/>
-      <c r="K49" s="26"/>
-      <c r="L49" s="26"/>
-      <c r="M49" s="26"/>
+      <c r="K49" s="28"/>
+      <c r="L49" s="28"/>
+      <c r="M49" s="28"/>
       <c r="N49" s="21"/>
       <c r="O49" s="21"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="25"/>
-      <c r="B50" s="26"/>
-      <c r="C50" s="26"/>
-      <c r="D50" s="26"/>
-      <c r="E50" s="26"/>
-      <c r="F50" s="26"/>
+      <c r="B50" s="28"/>
+      <c r="C50" s="28"/>
+      <c r="D50" s="28"/>
+      <c r="E50" s="28"/>
+      <c r="F50" s="28"/>
       <c r="J50" s="25"/>
-      <c r="K50" s="26"/>
-      <c r="L50" s="26"/>
-      <c r="M50" s="26"/>
+      <c r="K50" s="28"/>
+      <c r="L50" s="28"/>
+      <c r="M50" s="28"/>
       <c r="N50" s="21"/>
       <c r="O50" s="21"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="25"/>
-      <c r="B51" s="26"/>
-      <c r="C51" s="26"/>
-      <c r="D51" s="26"/>
-      <c r="E51" s="26"/>
-      <c r="F51" s="26"/>
+      <c r="B51" s="28"/>
+      <c r="C51" s="28"/>
+      <c r="D51" s="28"/>
+      <c r="E51" s="28"/>
+      <c r="F51" s="28"/>
       <c r="J51" s="25"/>
-      <c r="K51" s="26"/>
-      <c r="L51" s="26"/>
-      <c r="M51" s="26"/>
+      <c r="K51" s="28"/>
+      <c r="L51" s="28"/>
+      <c r="M51" s="28"/>
       <c r="N51" s="21"/>
       <c r="O51" s="21"/>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="25"/>
-      <c r="B52" s="26"/>
-      <c r="C52" s="26"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="26"/>
-      <c r="F52" s="26"/>
+      <c r="B52" s="28"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="28"/>
+      <c r="E52" s="28"/>
+      <c r="F52" s="28"/>
       <c r="J52" s="25"/>
-      <c r="K52" s="26"/>
-      <c r="L52" s="26"/>
-      <c r="M52" s="26"/>
+      <c r="K52" s="28"/>
+      <c r="L52" s="28"/>
+      <c r="M52" s="28"/>
       <c r="N52" s="21"/>
       <c r="O52" s="21"/>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="25"/>
-      <c r="B53" s="26"/>
-      <c r="C53" s="26"/>
-      <c r="D53" s="26"/>
-      <c r="E53" s="26"/>
-      <c r="F53" s="26"/>
+      <c r="B53" s="28"/>
+      <c r="C53" s="28"/>
+      <c r="D53" s="28"/>
+      <c r="E53" s="28"/>
+      <c r="F53" s="28"/>
       <c r="J53" s="25"/>
-      <c r="K53" s="26"/>
-      <c r="L53" s="26"/>
-      <c r="M53" s="26"/>
+      <c r="K53" s="28"/>
+      <c r="L53" s="28"/>
+      <c r="M53" s="28"/>
       <c r="N53" s="21"/>
       <c r="O53" s="21"/>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="25"/>
-      <c r="B54" s="26"/>
-      <c r="C54" s="26"/>
-      <c r="D54" s="26"/>
-      <c r="E54" s="26"/>
-      <c r="F54" s="26"/>
+      <c r="B54" s="28"/>
+      <c r="C54" s="28"/>
+      <c r="D54" s="28"/>
+      <c r="E54" s="28"/>
+      <c r="F54" s="28"/>
       <c r="J54" s="25"/>
-      <c r="K54" s="26"/>
-      <c r="L54" s="26"/>
-      <c r="M54" s="26"/>
+      <c r="K54" s="28"/>
+      <c r="L54" s="28"/>
+      <c r="M54" s="28"/>
       <c r="N54" s="21"/>
       <c r="O54" s="21"/>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="25"/>
-      <c r="B55" s="26"/>
-      <c r="C55" s="26"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="26"/>
-      <c r="F55" s="26"/>
+      <c r="B55" s="28"/>
+      <c r="C55" s="28"/>
+      <c r="D55" s="28"/>
+      <c r="E55" s="28"/>
+      <c r="F55" s="28"/>
       <c r="J55" s="25"/>
-      <c r="K55" s="26"/>
-      <c r="L55" s="26"/>
-      <c r="M55" s="26"/>
+      <c r="K55" s="28"/>
+      <c r="L55" s="28"/>
+      <c r="M55" s="28"/>
       <c r="N55" s="21"/>
       <c r="O55" s="21"/>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="25"/>
-      <c r="B56" s="26"/>
-      <c r="C56" s="26"/>
-      <c r="D56" s="26"/>
-      <c r="E56" s="26"/>
-      <c r="F56" s="26"/>
+      <c r="B56" s="28"/>
+      <c r="C56" s="28"/>
+      <c r="D56" s="28"/>
+      <c r="E56" s="28"/>
+      <c r="F56" s="28"/>
       <c r="J56" s="25"/>
-      <c r="K56" s="26"/>
-      <c r="L56" s="26"/>
-      <c r="M56" s="26"/>
+      <c r="K56" s="28"/>
+      <c r="L56" s="28"/>
+      <c r="M56" s="28"/>
       <c r="N56" s="21"/>
       <c r="O56" s="21"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="25"/>
-      <c r="B57" s="26"/>
-      <c r="C57" s="26"/>
-      <c r="D57" s="26"/>
-      <c r="E57" s="26"/>
-      <c r="F57" s="26"/>
+      <c r="B57" s="28"/>
+      <c r="C57" s="28"/>
+      <c r="D57" s="28"/>
+      <c r="E57" s="28"/>
+      <c r="F57" s="28"/>
       <c r="J57" s="25"/>
-      <c r="K57" s="26"/>
-      <c r="L57" s="26"/>
-      <c r="M57" s="26"/>
+      <c r="K57" s="28"/>
+      <c r="L57" s="28"/>
+      <c r="M57" s="28"/>
       <c r="N57" s="21"/>
       <c r="O57" s="21"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="25"/>
-      <c r="B58" s="26"/>
-      <c r="C58" s="26"/>
-      <c r="D58" s="26"/>
-      <c r="E58" s="26"/>
-      <c r="F58" s="26"/>
+      <c r="B58" s="28"/>
+      <c r="C58" s="28"/>
+      <c r="D58" s="28"/>
+      <c r="E58" s="28"/>
+      <c r="F58" s="28"/>
       <c r="J58" s="25"/>
-      <c r="K58" s="26"/>
-      <c r="L58" s="26"/>
-      <c r="M58" s="26"/>
+      <c r="K58" s="28"/>
+      <c r="L58" s="28"/>
+      <c r="M58" s="28"/>
       <c r="N58" s="21"/>
       <c r="O58" s="21"/>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="25"/>
-      <c r="B59" s="26"/>
-      <c r="C59" s="26"/>
-      <c r="D59" s="26"/>
-      <c r="E59" s="26"/>
-      <c r="F59" s="26"/>
+      <c r="B59" s="28"/>
+      <c r="C59" s="28"/>
+      <c r="D59" s="28"/>
+      <c r="E59" s="28"/>
+      <c r="F59" s="28"/>
       <c r="J59" s="25"/>
-      <c r="K59" s="26"/>
-      <c r="L59" s="26"/>
-      <c r="M59" s="26"/>
+      <c r="K59" s="28"/>
+      <c r="L59" s="28"/>
+      <c r="M59" s="28"/>
       <c r="N59" s="21"/>
       <c r="O59" s="21"/>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="25"/>
-      <c r="B60" s="26"/>
-      <c r="C60" s="26"/>
-      <c r="D60" s="26"/>
-      <c r="E60" s="26"/>
-      <c r="F60" s="26"/>
+      <c r="B60" s="28"/>
+      <c r="C60" s="28"/>
+      <c r="D60" s="28"/>
+      <c r="E60" s="28"/>
+      <c r="F60" s="28"/>
       <c r="J60" s="25"/>
-      <c r="K60" s="26"/>
-      <c r="L60" s="26"/>
-      <c r="M60" s="26"/>
+      <c r="K60" s="28"/>
+      <c r="L60" s="28"/>
+      <c r="M60" s="28"/>
       <c r="N60" s="21"/>
       <c r="O60" s="21"/>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="25"/>
-      <c r="B61" s="26"/>
-      <c r="C61" s="26"/>
-      <c r="D61" s="26"/>
-      <c r="E61" s="26"/>
-      <c r="F61" s="26"/>
+      <c r="B61" s="28"/>
+      <c r="C61" s="28"/>
+      <c r="D61" s="28"/>
+      <c r="E61" s="28"/>
+      <c r="F61" s="28"/>
       <c r="J61" s="25"/>
-      <c r="K61" s="26"/>
-      <c r="L61" s="26"/>
-      <c r="M61" s="26"/>
+      <c r="K61" s="28"/>
+      <c r="L61" s="28"/>
+      <c r="M61" s="28"/>
       <c r="N61" s="21"/>
       <c r="O61" s="21"/>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="25"/>
-      <c r="B62" s="26"/>
-      <c r="C62" s="26"/>
-      <c r="D62" s="26"/>
-      <c r="E62" s="26"/>
-      <c r="F62" s="26"/>
+      <c r="B62" s="28"/>
+      <c r="C62" s="28"/>
+      <c r="D62" s="28"/>
+      <c r="E62" s="28"/>
+      <c r="F62" s="28"/>
       <c r="J62" s="25"/>
-      <c r="K62" s="26"/>
-      <c r="L62" s="26"/>
-      <c r="M62" s="26"/>
+      <c r="K62" s="28"/>
+      <c r="L62" s="28"/>
+      <c r="M62" s="28"/>
       <c r="N62" s="21"/>
       <c r="O62" s="21"/>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="25"/>
-      <c r="B63" s="26"/>
-      <c r="C63" s="26"/>
-      <c r="D63" s="26"/>
-      <c r="E63" s="26"/>
-      <c r="F63" s="26"/>
+      <c r="B63" s="28"/>
+      <c r="C63" s="28"/>
+      <c r="D63" s="28"/>
+      <c r="E63" s="28"/>
+      <c r="F63" s="28"/>
       <c r="J63" s="25"/>
-      <c r="K63" s="26"/>
-      <c r="L63" s="26"/>
-      <c r="M63" s="26"/>
+      <c r="K63" s="28"/>
+      <c r="L63" s="28"/>
+      <c r="M63" s="28"/>
       <c r="N63" s="21"/>
       <c r="O63" s="21"/>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="25"/>
-      <c r="B64" s="26"/>
-      <c r="C64" s="26"/>
-      <c r="D64" s="26"/>
-      <c r="E64" s="26"/>
-      <c r="F64" s="26"/>
+      <c r="B64" s="28"/>
+      <c r="C64" s="28"/>
+      <c r="D64" s="28"/>
+      <c r="E64" s="28"/>
+      <c r="F64" s="28"/>
       <c r="J64" s="25"/>
-      <c r="K64" s="26"/>
-      <c r="L64" s="26"/>
-      <c r="M64" s="26"/>
+      <c r="K64" s="28"/>
+      <c r="L64" s="28"/>
+      <c r="M64" s="28"/>
       <c r="N64" s="21"/>
       <c r="O64" s="21"/>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="25"/>
-      <c r="B65" s="26"/>
-      <c r="C65" s="26"/>
-      <c r="D65" s="26"/>
-      <c r="E65" s="26"/>
-      <c r="F65" s="26"/>
+      <c r="B65" s="28"/>
+      <c r="C65" s="28"/>
+      <c r="D65" s="28"/>
+      <c r="E65" s="28"/>
+      <c r="F65" s="28"/>
       <c r="J65" s="25"/>
-      <c r="K65" s="26"/>
-      <c r="L65" s="26"/>
-      <c r="M65" s="26"/>
+      <c r="K65" s="28"/>
+      <c r="L65" s="28"/>
+      <c r="M65" s="28"/>
       <c r="N65" s="21"/>
       <c r="O65" s="21"/>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="25"/>
-      <c r="B66" s="26"/>
-      <c r="C66" s="26"/>
-      <c r="D66" s="26"/>
-      <c r="E66" s="26"/>
-      <c r="F66" s="26"/>
+      <c r="B66" s="28"/>
+      <c r="C66" s="28"/>
+      <c r="D66" s="28"/>
+      <c r="E66" s="28"/>
+      <c r="F66" s="28"/>
       <c r="J66" s="25"/>
-      <c r="K66" s="26"/>
-      <c r="L66" s="26"/>
-      <c r="M66" s="26"/>
+      <c r="K66" s="28"/>
+      <c r="L66" s="28"/>
+      <c r="M66" s="28"/>
       <c r="N66" s="21"/>
       <c r="O66" s="21"/>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="25"/>
-      <c r="B67" s="26"/>
-      <c r="C67" s="26"/>
-      <c r="D67" s="26"/>
-      <c r="E67" s="26"/>
-      <c r="F67" s="26"/>
+      <c r="B67" s="28"/>
+      <c r="C67" s="28"/>
+      <c r="D67" s="28"/>
+      <c r="E67" s="28"/>
+      <c r="F67" s="28"/>
       <c r="J67" s="25"/>
-      <c r="K67" s="26"/>
-      <c r="L67" s="26"/>
-      <c r="M67" s="26"/>
+      <c r="K67" s="28"/>
+      <c r="L67" s="28"/>
+      <c r="M67" s="28"/>
       <c r="N67" s="21"/>
       <c r="O67" s="21"/>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="25"/>
-      <c r="B68" s="26"/>
-      <c r="C68" s="26"/>
-      <c r="D68" s="26"/>
-      <c r="E68" s="26"/>
-      <c r="F68" s="26"/>
+      <c r="B68" s="28"/>
+      <c r="C68" s="28"/>
+      <c r="D68" s="28"/>
+      <c r="E68" s="28"/>
+      <c r="F68" s="28"/>
       <c r="J68" s="25"/>
-      <c r="K68" s="26"/>
-      <c r="L68" s="26"/>
-      <c r="M68" s="26"/>
+      <c r="K68" s="28"/>
+      <c r="L68" s="28"/>
+      <c r="M68" s="28"/>
       <c r="N68" s="21"/>
       <c r="O68" s="21"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="25"/>
-      <c r="B69" s="26"/>
-      <c r="C69" s="26"/>
-      <c r="D69" s="26"/>
-      <c r="E69" s="26"/>
-      <c r="F69" s="26"/>
+      <c r="B69" s="28"/>
+      <c r="C69" s="28"/>
+      <c r="D69" s="28"/>
+      <c r="E69" s="28"/>
+      <c r="F69" s="28"/>
       <c r="J69" s="25"/>
-      <c r="K69" s="26"/>
-      <c r="L69" s="26"/>
-      <c r="M69" s="26"/>
+      <c r="K69" s="28"/>
+      <c r="L69" s="28"/>
+      <c r="M69" s="28"/>
       <c r="N69" s="21"/>
       <c r="O69" s="21"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="25"/>
-      <c r="B70" s="26"/>
-      <c r="C70" s="26"/>
-      <c r="D70" s="26"/>
-      <c r="E70" s="26"/>
-      <c r="F70" s="26"/>
+      <c r="B70" s="28"/>
+      <c r="C70" s="28"/>
+      <c r="D70" s="28"/>
+      <c r="E70" s="28"/>
+      <c r="F70" s="28"/>
       <c r="J70" s="25"/>
-      <c r="K70" s="26"/>
-      <c r="L70" s="26"/>
-      <c r="M70" s="26"/>
+      <c r="K70" s="28"/>
+      <c r="L70" s="28"/>
+      <c r="M70" s="28"/>
       <c r="N70" s="21"/>
       <c r="O70" s="21"/>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="25"/>
-      <c r="B71" s="26"/>
-      <c r="C71" s="26"/>
-      <c r="D71" s="26"/>
-      <c r="E71" s="26"/>
-      <c r="F71" s="26"/>
+      <c r="B71" s="28"/>
+      <c r="C71" s="28"/>
+      <c r="D71" s="28"/>
+      <c r="E71" s="28"/>
+      <c r="F71" s="28"/>
       <c r="J71" s="25"/>
-      <c r="K71" s="26"/>
-      <c r="L71" s="26"/>
-      <c r="M71" s="26"/>
+      <c r="K71" s="28"/>
+      <c r="L71" s="28"/>
+      <c r="M71" s="28"/>
       <c r="N71" s="21"/>
       <c r="O71" s="21"/>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="25"/>
-      <c r="B72" s="26"/>
-      <c r="C72" s="26"/>
-      <c r="D72" s="26"/>
-      <c r="E72" s="26"/>
-      <c r="F72" s="26"/>
+      <c r="B72" s="28"/>
+      <c r="C72" s="28"/>
+      <c r="D72" s="28"/>
+      <c r="E72" s="28"/>
+      <c r="F72" s="28"/>
       <c r="J72" s="25"/>
-      <c r="K72" s="26"/>
-      <c r="L72" s="26"/>
-      <c r="M72" s="26"/>
+      <c r="K72" s="28"/>
+      <c r="L72" s="28"/>
+      <c r="M72" s="28"/>
       <c r="N72" s="21"/>
       <c r="O72" s="21"/>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="25"/>
-      <c r="B73" s="26"/>
-      <c r="C73" s="26"/>
-      <c r="D73" s="26"/>
-      <c r="E73" s="26"/>
-      <c r="F73" s="26"/>
+      <c r="B73" s="28"/>
+      <c r="C73" s="28"/>
+      <c r="D73" s="28"/>
+      <c r="E73" s="28"/>
+      <c r="F73" s="28"/>
       <c r="J73" s="25"/>
-      <c r="K73" s="26"/>
-      <c r="L73" s="26"/>
-      <c r="M73" s="26"/>
+      <c r="K73" s="28"/>
+      <c r="L73" s="28"/>
+      <c r="M73" s="28"/>
       <c r="N73" s="21"/>
       <c r="O73" s="21"/>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="25"/>
-      <c r="B74" s="26"/>
-      <c r="C74" s="26"/>
-      <c r="D74" s="26"/>
-      <c r="E74" s="26"/>
-      <c r="F74" s="26"/>
+      <c r="B74" s="28"/>
+      <c r="C74" s="28"/>
+      <c r="D74" s="28"/>
+      <c r="E74" s="28"/>
+      <c r="F74" s="28"/>
       <c r="J74" s="25"/>
-      <c r="K74" s="26"/>
-      <c r="L74" s="26"/>
-      <c r="M74" s="26"/>
+      <c r="K74" s="28"/>
+      <c r="L74" s="28"/>
+      <c r="M74" s="28"/>
       <c r="N74" s="21"/>
       <c r="O74" s="21"/>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" s="25"/>
-      <c r="B75" s="26"/>
-      <c r="C75" s="26"/>
-      <c r="D75" s="26"/>
-      <c r="E75" s="26"/>
-      <c r="F75" s="26"/>
+      <c r="B75" s="28"/>
+      <c r="C75" s="28"/>
+      <c r="D75" s="28"/>
+      <c r="E75" s="28"/>
+      <c r="F75" s="28"/>
       <c r="J75" s="25"/>
-      <c r="K75" s="26"/>
-      <c r="L75" s="26"/>
-      <c r="M75" s="26"/>
+      <c r="K75" s="28"/>
+      <c r="L75" s="28"/>
+      <c r="M75" s="28"/>
       <c r="N75" s="21"/>
       <c r="O75" s="21"/>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A76" s="25"/>
-      <c r="B76" s="26"/>
-      <c r="C76" s="26"/>
-      <c r="D76" s="26"/>
-      <c r="E76" s="26"/>
-      <c r="F76" s="26"/>
+      <c r="B76" s="28"/>
+      <c r="C76" s="28"/>
+      <c r="D76" s="28"/>
+      <c r="E76" s="28"/>
+      <c r="F76" s="28"/>
       <c r="J76" s="25"/>
-      <c r="K76" s="26"/>
-      <c r="L76" s="26"/>
-      <c r="M76" s="26"/>
+      <c r="K76" s="28"/>
+      <c r="L76" s="28"/>
+      <c r="M76" s="28"/>
       <c r="N76" s="21"/>
       <c r="O76" s="21"/>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A77" s="25"/>
-      <c r="B77" s="26"/>
-      <c r="C77" s="26"/>
-      <c r="D77" s="26"/>
-      <c r="E77" s="26"/>
-      <c r="F77" s="26"/>
+      <c r="B77" s="28"/>
+      <c r="C77" s="28"/>
+      <c r="D77" s="28"/>
+      <c r="E77" s="28"/>
+      <c r="F77" s="28"/>
       <c r="J77" s="25"/>
-      <c r="K77" s="26"/>
-      <c r="L77" s="26"/>
-      <c r="M77" s="26"/>
+      <c r="K77" s="28"/>
+      <c r="L77" s="28"/>
+      <c r="M77" s="28"/>
       <c r="N77" s="21"/>
       <c r="O77" s="21"/>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A78" s="25"/>
-      <c r="B78" s="26"/>
-      <c r="C78" s="26"/>
-      <c r="D78" s="26"/>
-      <c r="E78" s="26"/>
-      <c r="F78" s="26"/>
+      <c r="B78" s="28"/>
+      <c r="C78" s="28"/>
+      <c r="D78" s="28"/>
+      <c r="E78" s="28"/>
+      <c r="F78" s="28"/>
       <c r="J78" s="25"/>
-      <c r="K78" s="26"/>
-      <c r="L78" s="26"/>
-      <c r="M78" s="26"/>
+      <c r="K78" s="28"/>
+      <c r="L78" s="28"/>
+      <c r="M78" s="28"/>
       <c r="N78" s="21"/>
       <c r="O78" s="21"/>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A79" s="25"/>
-      <c r="B79" s="26"/>
-      <c r="C79" s="26"/>
-      <c r="D79" s="26"/>
-      <c r="E79" s="26"/>
-      <c r="F79" s="26"/>
+      <c r="B79" s="28"/>
+      <c r="C79" s="28"/>
+      <c r="D79" s="28"/>
+      <c r="E79" s="28"/>
+      <c r="F79" s="28"/>
       <c r="J79" s="25"/>
-      <c r="K79" s="26"/>
-      <c r="L79" s="26"/>
-      <c r="M79" s="26"/>
+      <c r="K79" s="28"/>
+      <c r="L79" s="28"/>
+      <c r="M79" s="28"/>
       <c r="N79" s="21"/>
       <c r="O79" s="21"/>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A80" s="25"/>
-      <c r="B80" s="26"/>
-      <c r="C80" s="26"/>
-      <c r="D80" s="26"/>
-      <c r="E80" s="26"/>
-      <c r="F80" s="26"/>
+      <c r="B80" s="28"/>
+      <c r="C80" s="28"/>
+      <c r="D80" s="28"/>
+      <c r="E80" s="28"/>
+      <c r="F80" s="28"/>
       <c r="J80" s="25"/>
-      <c r="K80" s="26"/>
-      <c r="L80" s="26"/>
-      <c r="M80" s="26"/>
+      <c r="K80" s="28"/>
+      <c r="L80" s="28"/>
+      <c r="M80" s="28"/>
       <c r="N80" s="21"/>
       <c r="O80" s="21"/>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" s="25"/>
-      <c r="B81" s="26"/>
-      <c r="C81" s="26"/>
-      <c r="D81" s="26"/>
-      <c r="E81" s="26"/>
-      <c r="F81" s="26"/>
+      <c r="B81" s="28"/>
+      <c r="C81" s="28"/>
+      <c r="D81" s="28"/>
+      <c r="E81" s="28"/>
+      <c r="F81" s="28"/>
       <c r="J81" s="25"/>
-      <c r="K81" s="26"/>
-      <c r="L81" s="26"/>
-      <c r="M81" s="26"/>
+      <c r="K81" s="28"/>
+      <c r="L81" s="28"/>
+      <c r="M81" s="28"/>
       <c r="N81" s="21"/>
       <c r="O81" s="21"/>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A82" s="25"/>
-      <c r="B82" s="26"/>
-      <c r="C82" s="26"/>
-      <c r="D82" s="26"/>
-      <c r="E82" s="26"/>
-      <c r="F82" s="26"/>
+      <c r="B82" s="28"/>
+      <c r="C82" s="28"/>
+      <c r="D82" s="28"/>
+      <c r="E82" s="28"/>
+      <c r="F82" s="28"/>
       <c r="J82" s="25"/>
-      <c r="K82" s="26"/>
-      <c r="L82" s="26"/>
-      <c r="M82" s="26"/>
+      <c r="K82" s="28"/>
+      <c r="L82" s="28"/>
+      <c r="M82" s="28"/>
       <c r="N82" s="21"/>
       <c r="O82" s="21"/>
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A83" s="25"/>
-      <c r="B83" s="26"/>
-      <c r="C83" s="26"/>
-      <c r="D83" s="26"/>
-      <c r="E83" s="26"/>
-      <c r="F83" s="26"/>
+      <c r="B83" s="28"/>
+      <c r="C83" s="28"/>
+      <c r="D83" s="28"/>
+      <c r="E83" s="28"/>
+      <c r="F83" s="28"/>
       <c r="J83" s="25"/>
-      <c r="K83" s="26"/>
-      <c r="L83" s="26"/>
-      <c r="M83" s="26"/>
+      <c r="K83" s="28"/>
+      <c r="L83" s="28"/>
+      <c r="M83" s="28"/>
       <c r="N83" s="21"/>
       <c r="O83" s="21"/>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A84" s="25"/>
-      <c r="B84" s="26"/>
-      <c r="C84" s="26"/>
-      <c r="D84" s="26"/>
-      <c r="E84" s="26"/>
-      <c r="F84" s="26"/>
+      <c r="B84" s="28"/>
+      <c r="C84" s="28"/>
+      <c r="D84" s="28"/>
+      <c r="E84" s="28"/>
+      <c r="F84" s="28"/>
       <c r="J84" s="25"/>
-      <c r="K84" s="26"/>
-      <c r="L84" s="26"/>
-      <c r="M84" s="26"/>
+      <c r="K84" s="28"/>
+      <c r="L84" s="28"/>
+      <c r="M84" s="28"/>
       <c r="N84" s="21"/>
       <c r="O84" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="202">
+    <mergeCell ref="A83:F83"/>
+    <mergeCell ref="J83:M83"/>
+    <mergeCell ref="A84:F84"/>
+    <mergeCell ref="J84:M84"/>
+    <mergeCell ref="A80:F80"/>
+    <mergeCell ref="J80:M80"/>
+    <mergeCell ref="A81:F81"/>
+    <mergeCell ref="J81:M81"/>
+    <mergeCell ref="A82:F82"/>
+    <mergeCell ref="J82:M82"/>
+    <mergeCell ref="A77:F77"/>
+    <mergeCell ref="J77:M77"/>
+    <mergeCell ref="A78:F78"/>
+    <mergeCell ref="J78:M78"/>
+    <mergeCell ref="A79:F79"/>
+    <mergeCell ref="J79:M79"/>
+    <mergeCell ref="A74:F74"/>
+    <mergeCell ref="J74:M74"/>
+    <mergeCell ref="A75:F75"/>
+    <mergeCell ref="J75:M75"/>
+    <mergeCell ref="A76:F76"/>
+    <mergeCell ref="J76:M76"/>
+    <mergeCell ref="A71:F71"/>
+    <mergeCell ref="J71:M71"/>
+    <mergeCell ref="A72:F72"/>
+    <mergeCell ref="J72:M72"/>
+    <mergeCell ref="A73:F73"/>
+    <mergeCell ref="J73:M73"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="J68:M68"/>
+    <mergeCell ref="A69:F69"/>
+    <mergeCell ref="J69:M69"/>
+    <mergeCell ref="A70:F70"/>
+    <mergeCell ref="J70:M70"/>
+    <mergeCell ref="A65:F65"/>
+    <mergeCell ref="J65:M65"/>
+    <mergeCell ref="A66:F66"/>
+    <mergeCell ref="J66:M66"/>
+    <mergeCell ref="A67:F67"/>
+    <mergeCell ref="J67:M67"/>
+    <mergeCell ref="A62:F62"/>
+    <mergeCell ref="J62:M62"/>
+    <mergeCell ref="A63:F63"/>
+    <mergeCell ref="J63:M63"/>
+    <mergeCell ref="A64:F64"/>
+    <mergeCell ref="J64:M64"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="J59:M59"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="J60:M60"/>
+    <mergeCell ref="A61:F61"/>
+    <mergeCell ref="J61:M61"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="J56:M56"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="J57:M57"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="J58:M58"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="J53:M53"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="J54:M54"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="J55:M55"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="J50:M50"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="J51:M51"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="J52:M52"/>
+    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="J47:M47"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="J48:M48"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="J49:M49"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="J44:M44"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="J45:M45"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="J46:M46"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="J41:M41"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="J42:M42"/>
+    <mergeCell ref="A43:F43"/>
+    <mergeCell ref="J43:M43"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="J38:M38"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="J39:M39"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="J40:M40"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="J35:M35"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="J36:M36"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="J37:M37"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="J33:M33"/>
+    <mergeCell ref="Q33:T33"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="J34:M34"/>
+    <mergeCell ref="Q34:V34"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="J31:M31"/>
+    <mergeCell ref="Q31:T31"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="J32:M32"/>
+    <mergeCell ref="Q32:T32"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="J29:M29"/>
+    <mergeCell ref="Q29:T29"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="J30:M30"/>
+    <mergeCell ref="Q30:T30"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="J27:M27"/>
+    <mergeCell ref="Q27:T27"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="J28:M28"/>
+    <mergeCell ref="Q28:T28"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="J25:M25"/>
+    <mergeCell ref="Q25:T25"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="J26:M26"/>
+    <mergeCell ref="Q26:T26"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="J23:M23"/>
+    <mergeCell ref="Q23:T23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="J24:M24"/>
+    <mergeCell ref="Q24:T24"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="J21:M21"/>
+    <mergeCell ref="Q21:T21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="J22:M22"/>
+    <mergeCell ref="Q22:T22"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="J19:M19"/>
+    <mergeCell ref="Q19:T19"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="J20:M20"/>
+    <mergeCell ref="Q20:T20"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="J17:M17"/>
+    <mergeCell ref="Q17:T17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="J18:M18"/>
+    <mergeCell ref="Q18:T18"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="J15:M15"/>
+    <mergeCell ref="Q15:T15"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="J16:M16"/>
+    <mergeCell ref="Q16:T16"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="J13:M13"/>
+    <mergeCell ref="Q13:T13"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="J14:M14"/>
+    <mergeCell ref="Q14:T14"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="J11:M11"/>
+    <mergeCell ref="Q11:T11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="J12:M12"/>
+    <mergeCell ref="Q12:T12"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="J9:M9"/>
+    <mergeCell ref="Q9:T9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="J10:M10"/>
+    <mergeCell ref="Q10:T10"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="Q7:T7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="Q8:T8"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="Q5:T5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="J6:M6"/>
+    <mergeCell ref="Q6:T6"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="J3:M3"/>
     <mergeCell ref="Q3:T3"/>
@@ -6194,196 +7648,6 @@
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="J2:M2"/>
     <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="Q7:T7"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="Q8:T8"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="J5:M5"/>
-    <mergeCell ref="Q5:T5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="Q6:T6"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="J11:M11"/>
-    <mergeCell ref="Q11:T11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="J12:M12"/>
-    <mergeCell ref="Q12:T12"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="J9:M9"/>
-    <mergeCell ref="Q9:T9"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="J10:M10"/>
-    <mergeCell ref="Q10:T10"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="J15:M15"/>
-    <mergeCell ref="Q15:T15"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="J16:M16"/>
-    <mergeCell ref="Q16:T16"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="J13:M13"/>
-    <mergeCell ref="Q13:T13"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="J14:M14"/>
-    <mergeCell ref="Q14:T14"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="J19:M19"/>
-    <mergeCell ref="Q19:T19"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="J20:M20"/>
-    <mergeCell ref="Q20:T20"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="J17:M17"/>
-    <mergeCell ref="Q17:T17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="J18:M18"/>
-    <mergeCell ref="Q18:T18"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="J23:M23"/>
-    <mergeCell ref="Q23:T23"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="J24:M24"/>
-    <mergeCell ref="Q24:T24"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="J21:M21"/>
-    <mergeCell ref="Q21:T21"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="J22:M22"/>
-    <mergeCell ref="Q22:T22"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="J27:M27"/>
-    <mergeCell ref="Q27:T27"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="J28:M28"/>
-    <mergeCell ref="Q28:T28"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="J25:M25"/>
-    <mergeCell ref="Q25:T25"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="J26:M26"/>
-    <mergeCell ref="Q26:T26"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="J31:M31"/>
-    <mergeCell ref="Q31:T31"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="J32:M32"/>
-    <mergeCell ref="Q32:T32"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="J29:M29"/>
-    <mergeCell ref="Q29:T29"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="J30:M30"/>
-    <mergeCell ref="Q30:T30"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="J35:M35"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="J36:M36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="J37:M37"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="J33:M33"/>
-    <mergeCell ref="Q33:T33"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="J34:M34"/>
-    <mergeCell ref="Q34:V34"/>
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="J41:M41"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="J42:M42"/>
-    <mergeCell ref="A43:F43"/>
-    <mergeCell ref="J43:M43"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="J38:M38"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="J39:M39"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="J40:M40"/>
-    <mergeCell ref="A47:F47"/>
-    <mergeCell ref="J47:M47"/>
-    <mergeCell ref="A48:F48"/>
-    <mergeCell ref="J48:M48"/>
-    <mergeCell ref="A49:F49"/>
-    <mergeCell ref="J49:M49"/>
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="J44:M44"/>
-    <mergeCell ref="A45:F45"/>
-    <mergeCell ref="J45:M45"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="J46:M46"/>
-    <mergeCell ref="A53:F53"/>
-    <mergeCell ref="J53:M53"/>
-    <mergeCell ref="A54:F54"/>
-    <mergeCell ref="J54:M54"/>
-    <mergeCell ref="A55:F55"/>
-    <mergeCell ref="J55:M55"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="J50:M50"/>
-    <mergeCell ref="A51:F51"/>
-    <mergeCell ref="J51:M51"/>
-    <mergeCell ref="A52:F52"/>
-    <mergeCell ref="J52:M52"/>
-    <mergeCell ref="A59:F59"/>
-    <mergeCell ref="J59:M59"/>
-    <mergeCell ref="A60:F60"/>
-    <mergeCell ref="J60:M60"/>
-    <mergeCell ref="A61:F61"/>
-    <mergeCell ref="J61:M61"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="J56:M56"/>
-    <mergeCell ref="A57:F57"/>
-    <mergeCell ref="J57:M57"/>
-    <mergeCell ref="A58:F58"/>
-    <mergeCell ref="J58:M58"/>
-    <mergeCell ref="A65:F65"/>
-    <mergeCell ref="J65:M65"/>
-    <mergeCell ref="A66:F66"/>
-    <mergeCell ref="J66:M66"/>
-    <mergeCell ref="A67:F67"/>
-    <mergeCell ref="J67:M67"/>
-    <mergeCell ref="A62:F62"/>
-    <mergeCell ref="J62:M62"/>
-    <mergeCell ref="A63:F63"/>
-    <mergeCell ref="J63:M63"/>
-    <mergeCell ref="A64:F64"/>
-    <mergeCell ref="J64:M64"/>
-    <mergeCell ref="A71:F71"/>
-    <mergeCell ref="J71:M71"/>
-    <mergeCell ref="A72:F72"/>
-    <mergeCell ref="J72:M72"/>
-    <mergeCell ref="A73:F73"/>
-    <mergeCell ref="J73:M73"/>
-    <mergeCell ref="A68:F68"/>
-    <mergeCell ref="J68:M68"/>
-    <mergeCell ref="A69:F69"/>
-    <mergeCell ref="J69:M69"/>
-    <mergeCell ref="A70:F70"/>
-    <mergeCell ref="J70:M70"/>
-    <mergeCell ref="A77:F77"/>
-    <mergeCell ref="J77:M77"/>
-    <mergeCell ref="A78:F78"/>
-    <mergeCell ref="J78:M78"/>
-    <mergeCell ref="A79:F79"/>
-    <mergeCell ref="J79:M79"/>
-    <mergeCell ref="A74:F74"/>
-    <mergeCell ref="J74:M74"/>
-    <mergeCell ref="A75:F75"/>
-    <mergeCell ref="J75:M75"/>
-    <mergeCell ref="A76:F76"/>
-    <mergeCell ref="J76:M76"/>
-    <mergeCell ref="A83:F83"/>
-    <mergeCell ref="J83:M83"/>
-    <mergeCell ref="A84:F84"/>
-    <mergeCell ref="J84:M84"/>
-    <mergeCell ref="A80:F80"/>
-    <mergeCell ref="J80:M80"/>
-    <mergeCell ref="A81:F81"/>
-    <mergeCell ref="J81:M81"/>
-    <mergeCell ref="A82:F82"/>
-    <mergeCell ref="J82:M82"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>